<commit_message>
Automatizado: Base de datos actualizada por el servidor
</commit_message>
<xml_diff>
--- a/registro_normatividades.xlsx
+++ b/registro_normatividades.xlsx
@@ -439,10 +439,14 @@
           <t>Constitución Política de los Estados Unidos Mexicanos</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Descargado como Constitución Política de los Estados Unidos Mexicanos.docx</t>
+          <t>https://legislacion.scjn.gob.mx/Buscador/Paginas/wfResultados.aspx?q=Bum7LdQ0Dg535FX3lWpLYlUgXYTx8K90EoJIKNtiXcyrP+kcmMpIvp+tV2Ad0/ktekoUMHqDJwBEnPKRauXIePRd50INM332a2oBhcxvi4VU/qZpOXwcKa25bbDLXOEx7yEC5Urbzfi/rNElovBoL/Xc6G2VxB/bqvVEd559WEhMkNra+hKi+6ZwkguNFKsR/zERzTmeincw4SWhrrSyycf/Q2ZdQa47vfax6KvQjaucx+AYweCHl0HtzrEPlzfxZ3JbArzr1Fe8UrLXw0/2+HVn9GUOwpyseJPNDOQrVHHb4kY1upGSyvnRuWHDl61ZrQ+Cen6jORmdEGwg1LHOlCnuPGu3MARvGrae7Em04/fJ8DDDZZM9feaAZTGWUOHuENt2Kgs5Vo0u6TYbt+dFu7ufa29KoXAbmTJrawwkP0lItAXnzpCT+cyg7D7uJxwtViPC+Jj7hUziANGIiHfBIA0kAWqGwJCkJ5WMThC+OUU=</t>
         </is>
       </c>
     </row>

</xml_diff>